<commit_message>
post from excel fixed
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/PostDatabase.xlsx
+++ b/App/CLI-backend/databases/PostDatabase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\serba\AppData\Roaming\SPB_Data\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D00A0B-60CF-49B8-B7DA-6A4A876F5D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36E53F74-3515-4990-9054-DD51F8D85A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1896" yWindow="3288" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet0" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>ID</t>
   </si>
@@ -41,27 +41,6 @@
   </si>
   <si>
     <t>NSFW</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>admin</t>
-  </si>
-  <si>
-    <t>ndjasnd</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
-    <t>No image link</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>false</t>
   </si>
 </sst>
 </file>
@@ -433,16 +412,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -468,29 +447,6 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed post deletion bug
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/PostDatabase.xlsx
+++ b/App/CLI-backend/databases/PostDatabase.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\serba\AppData\Roaming\SPB_Data\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
     </mc:Choice>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>ID</t>
   </si>
@@ -41,12 +41,34 @@
   </si>
   <si>
     <t>NSFW</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Mihai14</t>
+  </si>
+  <si>
+    <t>MyTitle</t>
+  </si>
+  <si>
+    <t>MyPostContents</t>
+  </si>
+  <si>
+    <t>No image link</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>true</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -412,39 +434,62 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="7.2109375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="6.70703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="14.10546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.80859375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.0078125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="6.20703125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>6</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>